<commit_message>
auto: scan 2026-05-27 21:50 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -856,6 +856,63 @@
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t>2026-05-26T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2367287</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Seattle be 68°F or higher on May 29?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.9935</v>
+      </c>
+      <c r="H7" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.008500000000000001</v>
+      </c>
+      <c r="J7" t="n">
+        <v>200</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-05-27T21:33:07.925460</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-05-29T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -936,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1151,6 +1208,36 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2367287</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.9935</v>
+      </c>
+      <c r="E7" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-05-29T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1162,7 +1249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1333,6 +1420,31 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2367287</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Seattle be 68°F or higher on</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.9935</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1486,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1558,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.1877</t>
+          <t>0.3220</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1733,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1951,6 +2063,34 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2367287</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Seattle be 68°F or higher on</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>74.09999999999999</v>
+      </c>
+      <c r="E7" t="n">
+        <v>96.45999999999999</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-05-28 22:04 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -913,6 +913,63 @@
       <c r="O7" t="inlineStr">
         <is>
           <t>2026-05-29T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2376000</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 72°F or higher on May 30?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.7122000000000001</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.4772</v>
+      </c>
+      <c r="H8" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="J8" t="n">
+        <v>200</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-05-28T21:53:44.774631</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-05-30T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -993,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1238,6 +1295,36 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2376000</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.7122000000000001</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.4772</v>
+      </c>
+      <c r="E8" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-05-30T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1249,7 +1336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1443,6 +1530,31 @@
         <v>0.9935</v>
       </c>
       <c r="G7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2376000</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 72°F or highe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.4772</v>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
@@ -1486,7 +1598,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1670,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3220</t>
+          <t>0.3442</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1845,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2091,6 +2203,34 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2376000</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 72°F or highe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>98.47</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-05-29 11:33 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,63 @@
         </is>
       </c>
       <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-05-30T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2375693</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Seattle be 63°F or below on May 30?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5683</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-0.2717</v>
+      </c>
+      <c r="H9" t="n">
+        <v>73</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="J9" t="n">
+        <v>200</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-05-29T10:41:36.642907</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>2026-05-30T12:00:00Z</t>
         </is>
@@ -1050,7 +1107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1325,6 +1382,36 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2375693</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.5683</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-0.2717</v>
+      </c>
+      <c r="E9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-30T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1336,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1557,6 +1644,31 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2375693</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Will the highest temperature in Seattle be 63°F or below on </t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>73</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.2717</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1710,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1782,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3442</t>
+          <t>0.3351</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1957,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1992,7 +2104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2231,6 +2343,34 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2375693</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Will the highest temperature in Seattle be 63°F or below on </t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>73</v>
+      </c>
+      <c r="E9" t="n">
+        <v>96.76000000000001</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-05-29 22:09 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -860,57 +860,63 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2367287</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Will the highest temperature in Seattle be 68°F or higher on May 29?</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="3" t="n">
         <v>0.0065</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="3" t="n">
         <v>0.9935</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="3" t="n">
         <v>74.09999999999999</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="3" t="n">
         <v>0.008500000000000001</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>23329.41</v>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>2026-05-27T21:33:07.925460</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>2026-05-29T12:00:00Z</t>
         </is>
@@ -1342,10 +1348,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>23329.41</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-05-29T12:00:00Z</t>
@@ -1687,7 +1695,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1722,7 +1730,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1742,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1766,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1778,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$9747.78</t>
+          <t>$33077.19</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1917,6 +1925,23 @@
       </c>
       <c r="E6" t="n">
         <v>0.0166</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>33077.19</v>
+      </c>
+      <c r="C7" t="n">
+        <v>43077.19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1934,7 +1959,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1969,7 +1994,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1981,7 +2006,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1993,7 +2018,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$9747.78</t>
+          <t>$33077.19</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2030,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$1949.56</t>
+          <t>$5512.87</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2042,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$4264.24</t>
+          <t>$8867.86</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2054,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.457</t>
+          <t>0.622</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2090,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>n=5 win_rate=20.0% total_pnl=$9747.78</t>
+          <t>n=6 win_rate=33.3% total_pnl=$33077.19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: scan 2026-05-30 10:04 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,12 +447,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -1033,6 +1033,63 @@
       <c r="O9" t="inlineStr">
         <is>
           <t>2026-05-30T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2383993</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in San Francisco be 70°F or higher on May 31?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.3972</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0.3428</v>
+      </c>
+      <c r="H10" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.262</v>
+      </c>
+      <c r="J10" t="n">
+        <v>200</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-05-30T09:26:27.387826</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2026-05-31T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1170,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1420,6 +1477,36 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2383993</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3972</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-0.3428</v>
+      </c>
+      <c r="E10" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-05-31T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1431,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1675,6 +1762,31 @@
         <v>-0.2717</v>
       </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2383993</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in San Francisco be 70°F or hig</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.3428</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>BUY_NO</t>
         </is>
@@ -1718,7 +1830,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1902,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3351</t>
+          <t>0.3360</t>
         </is>
       </c>
     </row>
@@ -1982,7 +2094,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2241,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -2396,6 +2508,34 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2383993</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in San Francisco be 70°F or hig</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>97.02</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-05-30 21:18 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1090,6 +1090,120 @@
       <c r="O10" t="inlineStr">
         <is>
           <t>2026-05-31T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2383715</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Atlanta be 76°F or higher on May 31?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.6241</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.1741</v>
+      </c>
+      <c r="H11" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.452</v>
+      </c>
+      <c r="J11" t="n">
+        <v>200</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-05-30T20:19:34.084717</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2026-05-31T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or higher on June 1?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.8511</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.5711000000000001</v>
+      </c>
+      <c r="H12" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J12" t="n">
+        <v>200</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-05-30T21:04:49.942326</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2026-06-01T12:00:00Z</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1507,6 +1621,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2383715</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.6241</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.1741</v>
+      </c>
+      <c r="E11" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-05-31T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.8511</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5711000000000001</v>
+      </c>
+      <c r="E12" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-06-01T12:00:00Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1518,7 +1692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1789,6 +1963,56 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2383715</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Atlanta be 76°F or higher on</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1741</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.5711000000000001</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
         </is>
       </c>
     </row>
@@ -1830,7 +2054,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -1902,7 +2126,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3360</t>
+          <t>0.3426</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2318,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2536,6 +2760,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2383715</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Atlanta be 76°F or higher on</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="E11" t="n">
+        <v>96.66</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="E12" t="n">
+        <v>96.72</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-05-30 21:40 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -463,7 +463,7 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -535,12 +535,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Entry Time</t>
+          <t>Entry Time (IL)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Resolution Date</t>
+          <t>Resolution Date (IL)</t>
         </is>
       </c>
     </row>
@@ -598,12 +598,12 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24T20:14:22.356082</t>
+          <t>2026-05-24 23:14</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25T12:00:00Z</t>
+          <t>2026-05-25 15:00</t>
         </is>
       </c>
     </row>
@@ -661,12 +661,12 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24T20:15:43.299202</t>
+          <t>2026-05-24 23:15</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25T12:00:00Z</t>
+          <t>2026-05-25 15:00</t>
         </is>
       </c>
     </row>
@@ -724,12 +724,12 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-24T20:20:15.757850</t>
+          <t>2026-05-24 23:20</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-25T12:00:00Z</t>
+          <t>2026-05-25 15:00</t>
         </is>
       </c>
     </row>
@@ -787,12 +787,12 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24T20:26:24.212548</t>
+          <t>2026-05-24 23:26</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26T12:00:00Z</t>
+          <t>2026-05-26 15:00</t>
         </is>
       </c>
     </row>
@@ -850,12 +850,12 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-24T20:27:49.936802</t>
+          <t>2026-05-24 23:27</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26T12:00:00Z</t>
+          <t>2026-05-26 15:00</t>
         </is>
       </c>
     </row>
@@ -913,12 +913,12 @@
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-27T21:33:07.925460</t>
+          <t>2026-05-28 00:33</t>
         </is>
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-29T12:00:00Z</t>
+          <t>2026-05-29 15:00</t>
         </is>
       </c>
     </row>
@@ -970,12 +970,12 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-05-28T21:53:44.774631</t>
+          <t>2026-05-29 00:53</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-05-30T12:00:00Z</t>
+          <t>2026-05-30 15:00</t>
         </is>
       </c>
     </row>
@@ -1027,12 +1027,12 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-05-29T10:41:36.642907</t>
+          <t>2026-05-29 13:41</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-05-30T12:00:00Z</t>
+          <t>2026-05-30 15:00</t>
         </is>
       </c>
     </row>
@@ -1084,12 +1084,12 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-05-30T09:26:27.387826</t>
+          <t>2026-05-30 12:26</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-05-31T12:00:00Z</t>
+          <t>2026-05-31 15:00</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1141,12 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-05-30T20:19:34.084717</t>
+          <t>2026-05-30 23:19</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-05-31T12:00:00Z</t>
+          <t>2026-05-31 15:00</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1198,12 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-05-30T21:04:49.942326</t>
+          <t>2026-05-31 00:04</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-06-01T12:00:00Z</t>
+          <t>2026-06-01 15:00</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Resolution Date</t>
+          <t>Resolution Date (IL)</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-25T12:00:00Z</t>
+          <t>2026-05-25 15:00</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-25T12:00:00Z</t>
+          <t>2026-05-25 15:00</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-05-25T12:00:00Z</t>
+          <t>2026-05-25 15:00</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-26T12:00:00Z</t>
+          <t>2026-05-26 15:00</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-26T12:00:00Z</t>
+          <t>2026-05-26 15:00</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-05-29T12:00:00Z</t>
+          <t>2026-05-29 15:00</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-05-30T12:00:00Z</t>
+          <t>2026-05-30 15:00</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-05-30T12:00:00Z</t>
+          <t>2026-05-30 15:00</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-05-31T12:00:00Z</t>
+          <t>2026-05-31 15:00</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-05-31T12:00:00Z</t>
+          <t>2026-05-31 15:00</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-06-01T12:00:00Z</t>
+          <t>2026-06-01 15:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: scan 2026-05-31 07:21 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -433,23 +433,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="11" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -527,6 +527,234 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Resolution Date (IL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or higher on June 1?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.8381999999999999</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.5482</v>
+      </c>
+      <c r="H2" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="J2" t="n">
+        <v>200</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:21</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2399769</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Chicago be 70°F or higher on June 2?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.6473</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.2877</v>
+      </c>
+      <c r="H3" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="J3" t="n">
+        <v>195.99</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:21</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2400000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Houston be 92°F or higher on June 2?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.4564</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.2814</v>
+      </c>
+      <c r="H4" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="J4" t="n">
+        <v>192.06</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:21</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2400011</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or higher on June 2?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.6432</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.4232</v>
+      </c>
+      <c r="H5" t="n">
+        <v>58</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="J5" t="n">
+        <v>188.22</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:21</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
         </is>
       </c>
     </row>
@@ -607,13 +835,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -659,6 +887,126 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Resolution Date (IL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.8381999999999999</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.5482</v>
+      </c>
+      <c r="E2" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2399769</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.6473</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.2877</v>
+      </c>
+      <c r="E3" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2400000</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.4564</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.2814</v>
+      </c>
+      <c r="E4" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2400011</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.6432</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.4232</v>
+      </c>
+      <c r="E5" t="n">
+        <v>58</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
         </is>
       </c>
     </row>
@@ -673,16 +1021,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -719,6 +1067,106 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5482</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2399769</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Chicago be 70°F or higher on</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-0.2877</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2400000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Houston be 92°F or higher on</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2814</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2400011</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>58</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.4232</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
         </is>
       </c>
     </row>
@@ -737,7 +1185,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -760,7 +1208,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -832,7 +1280,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0.3851</t>
         </is>
       </c>
     </row>
@@ -922,7 +1370,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1069,15 +1517,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1112,6 +1560,118 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2391532</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>89.84999999999999</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2399769</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Chicago be 70°F or higher on</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>65</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2400000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Houston be 92°F or higher on</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>65</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2400011</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>58</v>
+      </c>
+      <c r="E5" t="n">
+        <v>65</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-05-31 09:41 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -433,12 +433,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -755,6 +755,63 @@
       <c r="O5" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2391543</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in San Francisco be 68°F or higher on June 1?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.6805</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.2545</v>
+      </c>
+      <c r="H6" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.067</v>
+      </c>
+      <c r="J6" t="n">
+        <v>145.95</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-05-31 12:40</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:00</t>
         </is>
       </c>
     </row>
@@ -835,7 +892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1010,6 +1067,36 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2391543</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.6805</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.2545</v>
+      </c>
+      <c r="E6" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1021,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1167,6 +1254,31 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2391543</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in San Francisco be 68°F or hig</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.2545</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1320,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1392,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3851</t>
+          <t>0.3590</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1482,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1517,12 +1629,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
@@ -1672,6 +1784,34 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2391543</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in San Francisco be 68°F or hig</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>99.55</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: scan 2026-06-03 08:47 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -37,7 +37,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
         <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,11 +75,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -531,285 +545,315 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2391532</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Will the highest temperature in Los Angeles be 74°F or higher on June 1?</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
         <v>0.8381999999999999</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="2" t="n">
         <v>0.29</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="2" t="n">
         <v>0.5482</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="2" t="n">
         <v>65.7</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="2" t="n">
         <v>0.292</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>484.93</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>2026-05-31 10:21</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>2026-06-01 15:00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2399769</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Will the highest temperature in Chicago be 70°F or higher on June 2?</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Chicago</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>BUY_NO</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="2" t="n">
         <v>0.6473</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="2" t="n">
         <v>0.9350000000000001</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="2" t="n">
         <v>-0.2877</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="2" t="n">
         <v>57.4</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="2" t="n">
         <v>0.067</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" s="2" t="n">
         <v>195.99</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>2729.23</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>2026-05-31 10:21</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>2400000</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Will the highest temperature in Houston be 92°F or higher on June 2?</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Houston</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>0.4564</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="3" t="n">
         <v>0.175</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="3" t="n">
         <v>0.2814</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="3" t="n">
         <v>56.4</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="3" t="n">
         <v>0.177</v>
       </c>
-      <c r="J4" t="n">
+      <c r="J4" s="3" t="n">
         <v>192.06</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>-192.06</v>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>2026-05-31 10:21</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2400011</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Will the highest temperature in Los Angeles be 74°F or higher on June 2?</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="2" t="n">
         <v>0.6432</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="2" t="n">
         <v>0.22</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="2" t="n">
         <v>0.4232</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="2" t="n">
         <v>0.222</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="2" t="n">
         <v>188.22</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>659.62</v>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>2026-05-31 10:21</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2391543</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Will the highest temperature in San Francisco be 68°F or higher on June 1?</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>San Francisco</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>BUY_NO</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="2" t="n">
         <v>0.6805</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="2" t="n">
         <v>0.9350000000000001</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="2" t="n">
         <v>-0.2545</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="2" t="n">
         <v>67.3</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" s="2" t="n">
         <v>0.067</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J6" s="2" t="n">
         <v>145.95</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>2032.41</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>2026-05-31 12:40</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>2026-06-01 15:00</t>
         </is>
@@ -967,10 +1011,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>484.93</v>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>2026-06-01 15:00</t>
@@ -997,10 +1043,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>2729.23</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
@@ -1027,10 +1075,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>-192.06</v>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
@@ -1057,10 +1107,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>659.62</v>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
@@ -1087,10 +1139,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2032.41</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>2026-06-01 15:00</t>
@@ -1297,7 +1351,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1332,7 +1386,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1398,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1410,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1422,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1434,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$5714.13</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1442,6 +1496,91 @@
         <is>
           <t>Drawdown (%)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>484.93</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10484.93</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3214.17</v>
+      </c>
+      <c r="C3" t="n">
+        <v>13214.17</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3022.11</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13022.11</v>
+      </c>
+      <c r="D4" t="n">
+        <v>192.06</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0145</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>3681.72</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13681.72</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5714.13</v>
+      </c>
+      <c r="C6" t="n">
+        <v>15714.13</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1459,7 +1598,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1494,7 +1633,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1506,7 +1645,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>80.0%</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1657,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$5714.13</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1669,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$1142.83</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1681,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$1072.97</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1693,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>1.065</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1705,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>$0.00</t>
+          <t>$192.06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: scan 2026-06-03 11:50 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -856,6 +856,120 @@
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t>2026-06-01 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2416309</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or higher on June 4?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8921</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.6171</v>
+      </c>
+      <c r="H7" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.277</v>
+      </c>
+      <c r="J7" t="n">
+        <v>200</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:49</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2424766</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or higher on June 5?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.8423</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.5873</v>
+      </c>
+      <c r="H8" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.257</v>
+      </c>
+      <c r="J8" t="n">
+        <v>200</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-06-03 14:50</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-06-05 15:00</t>
         </is>
       </c>
     </row>
@@ -936,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1151,6 +1265,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2416309</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.8921</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.6171</v>
+      </c>
+      <c r="E7" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-06-04 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2424766</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.8423</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.255</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.5873</v>
+      </c>
+      <c r="E8" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-06-05 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1162,7 +1336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1333,6 +1507,56 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>BUY_NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2416309</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.6171</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2424766</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.5873</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1598,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1670,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.3590</t>
+          <t>0.4285</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1845,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1951,6 +2175,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2416309</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>99.23</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2424766</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Los Angeles be 74°F or highe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Los Angeles</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>99.56999999999999</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: resolve 2026-06-04 16:21 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -860,57 +860,63 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2416309</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Will the highest temperature in Los Angeles be 74°F or higher on June 4?</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="2" t="n">
         <v>0.8921</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="2" t="n">
         <v>0.275</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="2" t="n">
         <v>0.6171</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="2" t="n">
         <v>58.8</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="2" t="n">
         <v>0.277</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="2" t="n">
         <v>200</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>522.02</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>2026-06-03 14:49</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>2026-06-04 15:00</t>
         </is>
@@ -1285,10 +1291,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>522.02</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-06-04 15:00</t>
@@ -1610,7 +1618,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1630,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1654,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1666,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$5714.13</t>
+          <t>$6236.15</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1804,6 +1812,23 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>6236.15</v>
+      </c>
+      <c r="C7" t="n">
+        <v>16236.15</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1857,7 +1882,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1894,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1906,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$5714.13</t>
+          <t>$6236.15</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1918,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$1142.83</t>
+          <t>$1039.36</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1930,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$1072.97</t>
+          <t>$1006.43</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1942,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.065</t>
+          <t>1.033</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: scan 2026-06-05 10:40 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -52,14 +52,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -590,11 +590,11 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
-        <v>484.93</v>
+        <v>-200</v>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
@@ -653,81 +653,81 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>-195.99</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:21</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2400000</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Houston be 92°F or higher on June 2?</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.4564</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0.2814</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>192.06</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
           <t>False</t>
         </is>
       </c>
-      <c r="M3" s="2" t="n">
-        <v>2729.23</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="M4" s="2" t="n">
+        <v>-192.06</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>2026-05-31 10:21</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02 15:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>2400000</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Will the highest temperature in Houston be 92°F or higher on June 2?</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Houston</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>BUY_YES</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>0.4564</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>0.2814</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>56.4</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>0.177</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>192.06</v>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>-192.06</v>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-31 10:21</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>2026-06-02 15:00</t>
         </is>
@@ -779,11 +779,11 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
-        <v>659.62</v>
+        <v>-188.22</v>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
@@ -842,11 +842,11 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
-        <v>2032.41</v>
+        <v>-145.95</v>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
@@ -860,63 +860,63 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>2416309</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Will the highest temperature in Los Angeles be 74°F or higher on June 4?</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>0.8921</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>0.275</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="3" t="n">
         <v>0.6171</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="3" t="n">
         <v>58.8</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="3" t="n">
         <v>0.277</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="J7" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="M7" s="2" t="n">
+      <c r="M7" s="3" t="n">
         <v>522.02</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>2026-06-03 14:49</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O7" s="3" t="inlineStr">
         <is>
           <t>2026-06-04 15:00</t>
         </is>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$6236.15</t>
+          <t>$-400.20</t>
         </is>
       </c>
     </row>
@@ -1735,10 +1735,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>484.93</v>
+        <v>-200</v>
       </c>
       <c r="C2" t="n">
-        <v>10484.93</v>
+        <v>9800</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1752,16 +1752,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>3214.17</v>
+        <v>-395.99</v>
       </c>
       <c r="C3" t="n">
-        <v>13214.17</v>
+        <v>9604.01</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>195.99</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="4">
@@ -1769,16 +1769,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>3022.11</v>
+        <v>-588.05</v>
       </c>
       <c r="C4" t="n">
-        <v>13022.11</v>
+        <v>9411.950000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>192.06</v>
+        <v>388.05</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0145</v>
+        <v>0.0396</v>
       </c>
     </row>
     <row r="5">
@@ -1786,16 +1786,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>3681.72</v>
+        <v>-776.27</v>
       </c>
       <c r="C5" t="n">
-        <v>13681.72</v>
+        <v>9223.73</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>576.27</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>0.0588</v>
       </c>
     </row>
     <row r="6">
@@ -1803,16 +1803,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>5714.13</v>
+        <v>-922.22</v>
       </c>
       <c r="C6" t="n">
-        <v>15714.13</v>
+        <v>9077.780000000001</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>722.22</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>0.0737</v>
       </c>
     </row>
     <row r="7">
@@ -1820,16 +1820,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>6236.15</v>
+        <v>-400.2</v>
       </c>
       <c r="C7" t="n">
-        <v>16236.15</v>
+        <v>9599.799999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>200.2</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.0204</v>
       </c>
     </row>
   </sheetData>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>83.3%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$6236.15</t>
+          <t>$-400.20</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$1039.36</t>
+          <t>$-66.70</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$1006.43</t>
+          <t>$263.89</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1942,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1.033</t>
+          <t>-0.253</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>$192.06</t>
+          <t>$922.22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: resolve 2026-06-05 15:56 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -923,57 +923,63 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>2424766</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Will the highest temperature in Los Angeles be 74°F or higher on June 5?</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="3" t="n">
         <v>0.8423</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="3" t="n">
         <v>0.255</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="3" t="n">
         <v>0.5873</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="3" t="n">
         <v>56.5</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="3" t="n">
         <v>0.257</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>578.21</v>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
         <is>
           <t>2026-06-03 14:50</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>2026-06-05 15:00</t>
         </is>
@@ -1323,10 +1329,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>578.21</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>2026-06-05 15:00</t>
@@ -1583,7 +1591,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1618,7 +1626,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1638,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1662,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1674,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$-400.20</t>
+          <t>$178.01</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1830,6 +1838,23 @@
       </c>
       <c r="E7" t="n">
         <v>0.0204</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>178.01</v>
+      </c>
+      <c r="C8" t="n">
+        <v>10178.01</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1847,7 +1872,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1882,7 +1907,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1919,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1931,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$-400.20</t>
+          <t>$178.01</t>
         </is>
       </c>
     </row>
@@ -1918,7 +1943,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$-66.70</t>
+          <t>$25.43</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1955,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$263.89</t>
+          <t>$332.59</t>
         </is>
       </c>
     </row>
@@ -1942,7 +1967,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-0.253</t>
+          <t>0.076</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: scan 2026-07-21 09:20 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -982,6 +982,63 @@
       <c r="O8" s="3" t="inlineStr">
         <is>
           <t>2026-06-05 15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3009102</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Will the highest temperature in Denver be 94°F or higher on July 22?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3527</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1077</v>
+      </c>
+      <c r="H9" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="J9" t="n">
+        <v>75</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-07-21 12:20</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2026-07-22 15:00</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1341,6 +1398,36 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3009102</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3527</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1077</v>
+      </c>
+      <c r="E9" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-07-22 15:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1352,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1571,6 +1658,31 @@
         <v>0.5873</v>
       </c>
       <c r="G8" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3009102</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Will the highest temperature in Denver be 94°F or higher on </t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1077</v>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
@@ -1614,7 +1726,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1798,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.4285</t>
+          <t>0.3884</t>
         </is>
       </c>
     </row>
@@ -1895,7 +2007,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2281,6 +2393,34 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3009102</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Will the highest temperature in Denver be 94°F or higher on </t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>65</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>BUY_YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
auto: resolve 2026-07-22 15:06 UTC
</commit_message>
<xml_diff>
--- a/exports/weather_bot_report.xlsx
+++ b/exports/weather_bot_report.xlsx
@@ -986,57 +986,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>3009102</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Will the highest temperature in Denver be 94°F or higher on July 22?</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Denver</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>BUY_YES</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="3" t="n">
         <v>0.3527</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="3" t="n">
         <v>0.245</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="3" t="n">
         <v>0.1077</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="3" t="n">
         <v>67.2</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="3" t="n">
         <v>0.247</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>228.64</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
         <is>
           <t>2026-07-21 12:20</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>2026-07-22 15:00</t>
         </is>
@@ -1418,10 +1424,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PENDING</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>228.64</v>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>2026-07-22 15:00</t>
@@ -1738,7 +1746,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1758,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1782,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>37.5%</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1794,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$178.01</t>
+          <t>$406.66</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1966,6 +1974,23 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>406.66</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10406.66</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2019,7 +2044,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2056,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>37.5%</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2068,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>$178.01</t>
+          <t>$406.66</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2080,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$25.43</t>
+          <t>$50.83</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2092,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$332.59</t>
+          <t>$318.29</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2104,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.076</t>
+          <t>0.160</t>
         </is>
       </c>
     </row>

</xml_diff>